<commit_message>
Add subtotal rows for each category group
Inserts three subtotal rows (① 実験準備時間, ② 実験評価時間,
③ 波形作成・クライテリア確認時間) with aggregated hours and days,
styled in medium-blue to distinguish from data and TOTAL rows.

https://claude.ai/code/session_01W1qyWnBmW1iVnFoqFo3tKv
</commit_message>
<xml_diff>
--- a/QDC_FULL_schedule.xlsx
+++ b/QDC_FULL_schedule.xlsx
@@ -41,20 +41,20 @@
     </font>
     <font>
       <name val="Meiryo"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Meiryo"/>
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Meiryo"/>
       <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Meiryo"/>
+      <b val="1"/>
       <color rgb="00000000"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Meiryo"/>
@@ -68,7 +68,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +123,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B8CCE4"/>
       </patternFill>
     </fill>
   </fills>
@@ -232,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -240,34 +245,44 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -644,7 +659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -799,113 +814,179 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="24" customHeight="1">
       <c r="A7" s="10" t="n"/>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>① 実験準備時間 小計</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n"/>
+      <c r="D7" s="15" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>14.9</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>実験評価時間(h)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>CD実験・作業</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D8" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F8" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G8" s="9" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="11" t="inlineStr">
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>定置実験・作業</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D9" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E9" s="7" t="n">
         <v>0.75</v>
       </c>
-      <c r="F8" s="8" t="n">
+      <c r="F9" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="G8" s="9" t="n">
+      <c r="G9" s="9" t="n">
         <v>0.75</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>② 実験評価時間 小計</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>解析時間</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>波形作成、クライテリア確認時間(h)</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n"/>
-      <c r="D9" s="6" t="n">
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E11" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F11" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="G9" s="9" t="n">
+      <c r="G11" s="9" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>③ 波形作成・クライテリア確認時間 小計</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="G12" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D13" s="19" t="n">
         <v>44.9</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E13" s="20" t="n">
         <v>5.61</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="F13" s="19" t="n">
         <v>44.9</v>
       </c>
-      <c r="G10" s="16" t="n">
+      <c r="G13" s="20" t="n">
         <v>5.61</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>凡例：1日 = 8時間換算</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A10:C10"/>
+  <mergeCells count="11">
+    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A9"/>
-    <mergeCell ref="A3:A8"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="A3:A10"/>
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="B3:B6"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B12:C12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add reduction columns (削減時間h / 削減日数日)
Adds two columns showing manual minus auto for each row,
subtotal, and TOTAL — making automation savings immediately visible.

https://claude.ai/code/session_01W1qyWnBmW1iVnFoqFo3tKv
</commit_message>
<xml_diff>
--- a/QDC_FULL_schedule.xlsx
+++ b/QDC_FULL_schedule.xlsx
@@ -68,7 +68,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +118,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBE5D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -237,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -266,19 +276,25 @@
     <xf numFmtId="2" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -659,7 +675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,6 +685,8 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -718,6 +736,18 @@
 (日)</t>
         </is>
       </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>削減時間
+(h)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>削減日数
+(日)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -748,11 +778,17 @@
       <c r="G3" s="9" t="n">
         <v>0.15</v>
       </c>
+      <c r="H3" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="10" t="n"/>
-      <c r="B4" s="10" t="n"/>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="A4" s="12" t="n"/>
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>スタンバイ
 （C/D載せ・降ろし）</t>
@@ -770,10 +806,16 @@
       <c r="G4" s="9" t="n">
         <v>0.38</v>
       </c>
+      <c r="H4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="10" t="n"/>
-      <c r="B5" s="10" t="n"/>
+      <c r="A5" s="12" t="n"/>
+      <c r="B5" s="12" t="n"/>
       <c r="C5" s="5" t="inlineStr">
         <is>
           <t>計測準備
@@ -792,11 +834,17 @@
       <c r="G5" s="9" t="n">
         <v>1.19</v>
       </c>
+      <c r="H5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="10" t="n"/>
-      <c r="B6" s="12" t="n"/>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="n"/>
+      <c r="B6" s="14" t="n"/>
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>DTC取得</t>
         </is>
@@ -813,30 +861,42 @@
       <c r="G6" s="9" t="n">
         <v>0.15</v>
       </c>
+      <c r="H6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="10" t="n"/>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="A7" s="12" t="n"/>
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>① 実験準備時間 小計</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="15" t="n">
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="17" t="n">
         <v>14.9</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="18" t="n">
         <v>1.86</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="17" t="n">
         <v>14.9</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="G7" s="18" t="n">
         <v>1.86</v>
       </c>
+      <c r="H7" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="10" t="n"/>
+      <c r="A8" s="12" t="n"/>
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>実験評価時間(h)</t>
@@ -859,11 +919,17 @@
       <c r="G8" s="9" t="n">
         <v>1</v>
       </c>
+      <c r="H8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="12" t="n"/>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="14" t="n"/>
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>定置実験・作業</t>
         </is>
@@ -880,26 +946,38 @@
       <c r="G9" s="9" t="n">
         <v>0.75</v>
       </c>
+      <c r="H9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="12" t="n"/>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="n"/>
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>② 実験評価時間 小計</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="15" t="n">
+      <c r="C10" s="16" t="n"/>
+      <c r="D10" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="18" t="n">
         <v>1.75</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="F10" s="17" t="n">
         <v>14</v>
       </c>
-      <c r="G10" s="16" t="n">
+      <c r="G10" s="18" t="n">
         <v>1.75</v>
+      </c>
+      <c r="H10" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="36" customHeight="1">
@@ -913,7 +991,7 @@
           <t>波形作成、クライテリア確認時間(h)</t>
         </is>
       </c>
-      <c r="C11" s="17" t="n"/>
+      <c r="C11" s="19" t="n"/>
       <c r="D11" s="6" t="n">
         <v>16</v>
       </c>
@@ -926,49 +1004,67 @@
       <c r="G11" s="9" t="n">
         <v>2</v>
       </c>
+      <c r="H11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="n"/>
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>③ 波形作成・クライテリア確認時間 小計</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="15" t="n">
+      <c r="C12" s="16" t="n"/>
+      <c r="D12" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="G12" s="16" t="n">
+      <c r="G12" s="18" t="n">
         <v>2</v>
       </c>
+      <c r="H12" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="18" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="21" t="n">
         <v>44.9</v>
       </c>
-      <c r="E13" s="20" t="n">
+      <c r="E13" s="22" t="n">
         <v>5.61</v>
       </c>
-      <c r="F13" s="19" t="n">
+      <c r="F13" s="21" t="n">
         <v>44.9</v>
       </c>
-      <c r="G13" s="20" t="n">
+      <c r="G13" s="22" t="n">
         <v>5.61</v>
       </c>
+      <c r="H13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>凡例：1日 = 8時間換算</t>
         </is>
@@ -976,15 +1072,15 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A15:I15"/>
     <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="A3:A10"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A1:I1"/>
     <mergeCell ref="B3:B6"/>
     <mergeCell ref="B8:B9"/>
-    <mergeCell ref="A15:G15"/>
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="B12:C12"/>
   </mergeCells>

</xml_diff>